<commit_message>
Docs: add "Notes / Test result" column to feature list
Empty trailing column (CSV + xlsx) to fill in as you test each feature.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-feature-list.xlsx
+++ b/docs/finwise-feature-list.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:G73"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="26.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="56.83203125" customWidth="1"/>
     <col min="5" max="5" width="50.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,6 +427,9 @@
       <c r="F1" t="str">
         <v>Status</v>
       </c>
+      <c r="G1" t="str">
+        <v>Notes / Test result</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +450,9 @@
       <c r="F2" t="str">
         <v>Live</v>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,6 +473,9 @@
       <c r="F3" t="str">
         <v>Live</v>
       </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -486,6 +496,9 @@
       <c r="F4" t="str">
         <v>Live</v>
       </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -506,6 +519,9 @@
       <c r="F5" t="str">
         <v>Live</v>
       </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -525,6 +541,9 @@
       </c>
       <c r="F6" t="str">
         <v>Live</v>
+      </c>
+      <c r="G6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -546,6 +565,9 @@
       <c r="F7" t="str">
         <v>Live</v>
       </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -566,6 +588,9 @@
       <c r="F8" t="str">
         <v>Live</v>
       </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -586,6 +611,9 @@
       <c r="F9" t="str">
         <v>Live</v>
       </c>
+      <c r="G9" t="str">
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -606,6 +634,9 @@
       <c r="F10" t="str">
         <v>Live</v>
       </c>
+      <c r="G10" t="str">
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -626,6 +657,9 @@
       <c r="F11" t="str">
         <v>Live</v>
       </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -646,6 +680,9 @@
       <c r="F12" t="str">
         <v>Live</v>
       </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -666,6 +703,9 @@
       <c r="F13" t="str">
         <v>Live</v>
       </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -686,6 +726,9 @@
       <c r="F14" t="str">
         <v>Live</v>
       </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -706,6 +749,9 @@
       <c r="F15" t="str">
         <v>Live</v>
       </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -726,6 +772,9 @@
       <c r="F16" t="str">
         <v>Live</v>
       </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -746,6 +795,9 @@
       <c r="F17" t="str">
         <v>Live</v>
       </c>
+      <c r="G17" t="str">
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -766,6 +818,9 @@
       <c r="F18" t="str">
         <v>Live</v>
       </c>
+      <c r="G18" t="str">
+        <v/>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -786,6 +841,9 @@
       <c r="F19" t="str">
         <v>Live</v>
       </c>
+      <c r="G19" t="str">
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -806,6 +864,9 @@
       <c r="F20" t="str">
         <v>Live</v>
       </c>
+      <c r="G20" t="str">
+        <v/>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -826,6 +887,9 @@
       <c r="F21" t="str">
         <v>Live</v>
       </c>
+      <c r="G21" t="str">
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -845,6 +909,9 @@
       </c>
       <c r="F22" t="str">
         <v>Live</v>
+      </c>
+      <c r="G22" t="str">
+        <v/>
       </c>
     </row>
     <row r="23">
@@ -866,6 +933,9 @@
       <c r="F23" t="str">
         <v>Live</v>
       </c>
+      <c r="G23" t="str">
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -886,6 +956,9 @@
       <c r="F24" t="str">
         <v>Live</v>
       </c>
+      <c r="G24" t="str">
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -906,6 +979,9 @@
       <c r="F25" t="str">
         <v>Live</v>
       </c>
+      <c r="G25" t="str">
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -925,6 +1001,9 @@
       </c>
       <c r="F26" t="str">
         <v>Live</v>
+      </c>
+      <c r="G26" t="str">
+        <v/>
       </c>
     </row>
     <row r="27">
@@ -946,6 +1025,9 @@
       <c r="F27" t="str">
         <v>Live</v>
       </c>
+      <c r="G27" t="str">
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -966,6 +1048,9 @@
       <c r="F28" t="str">
         <v>Live</v>
       </c>
+      <c r="G28" t="str">
+        <v/>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -985,6 +1070,9 @@
       </c>
       <c r="F29" t="str">
         <v>Live</v>
+      </c>
+      <c r="G29" t="str">
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -1006,6 +1094,9 @@
       <c r="F30" t="str">
         <v>Live</v>
       </c>
+      <c r="G30" t="str">
+        <v/>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1026,6 +1117,9 @@
       <c r="F31" t="str">
         <v>Live</v>
       </c>
+      <c r="G31" t="str">
+        <v/>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1046,6 +1140,9 @@
       <c r="F32" t="str">
         <v>Live</v>
       </c>
+      <c r="G32" t="str">
+        <v/>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1066,6 +1163,9 @@
       <c r="F33" t="str">
         <v>Live</v>
       </c>
+      <c r="G33" t="str">
+        <v/>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -1086,6 +1186,9 @@
       <c r="F34" t="str">
         <v>Live</v>
       </c>
+      <c r="G34" t="str">
+        <v/>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -1106,6 +1209,9 @@
       <c r="F35" t="str">
         <v>Live</v>
       </c>
+      <c r="G35" t="str">
+        <v/>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -1126,6 +1232,9 @@
       <c r="F36" t="str">
         <v>Live</v>
       </c>
+      <c r="G36" t="str">
+        <v/>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
@@ -1145,6 +1254,9 @@
       </c>
       <c r="F37" t="str">
         <v>Coming soon</v>
+      </c>
+      <c r="G37" t="str">
+        <v/>
       </c>
     </row>
     <row r="38">
@@ -1166,6 +1278,9 @@
       <c r="F38" t="str">
         <v>Live</v>
       </c>
+      <c r="G38" t="str">
+        <v/>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
@@ -1186,6 +1301,9 @@
       <c r="F39" t="str">
         <v>Live</v>
       </c>
+      <c r="G39" t="str">
+        <v/>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -1206,6 +1324,9 @@
       <c r="F40" t="str">
         <v>Live</v>
       </c>
+      <c r="G40" t="str">
+        <v/>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -1226,6 +1347,9 @@
       <c r="F41" t="str">
         <v>Live</v>
       </c>
+      <c r="G41" t="str">
+        <v/>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -1246,6 +1370,9 @@
       <c r="F42" t="str">
         <v>Live</v>
       </c>
+      <c r="G42" t="str">
+        <v/>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -1266,6 +1393,9 @@
       <c r="F43" t="str">
         <v>Live</v>
       </c>
+      <c r="G43" t="str">
+        <v/>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -1285,6 +1415,9 @@
       </c>
       <c r="F44" t="str">
         <v>Live</v>
+      </c>
+      <c r="G44" t="str">
+        <v/>
       </c>
     </row>
     <row r="45">
@@ -1306,6 +1439,9 @@
       <c r="F45" t="str">
         <v>Live</v>
       </c>
+      <c r="G45" t="str">
+        <v/>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -1326,6 +1462,9 @@
       <c r="F46" t="str">
         <v>Live</v>
       </c>
+      <c r="G46" t="str">
+        <v/>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -1346,6 +1485,9 @@
       <c r="F47" t="str">
         <v>Live</v>
       </c>
+      <c r="G47" t="str">
+        <v/>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -1366,6 +1508,9 @@
       <c r="F48" t="str">
         <v>Live</v>
       </c>
+      <c r="G48" t="str">
+        <v/>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -1386,6 +1531,9 @@
       <c r="F49" t="str">
         <v>Live</v>
       </c>
+      <c r="G49" t="str">
+        <v/>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -1405,6 +1553,9 @@
       </c>
       <c r="F50" t="str">
         <v>Live</v>
+      </c>
+      <c r="G50" t="str">
+        <v/>
       </c>
     </row>
     <row r="51">
@@ -1426,6 +1577,9 @@
       <c r="F51" t="str">
         <v>Live</v>
       </c>
+      <c r="G51" t="str">
+        <v/>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
@@ -1446,6 +1600,9 @@
       <c r="F52" t="str">
         <v>Live</v>
       </c>
+      <c r="G52" t="str">
+        <v/>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="str">
@@ -1466,6 +1623,9 @@
       <c r="F53" t="str">
         <v>Live</v>
       </c>
+      <c r="G53" t="str">
+        <v/>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="str">
@@ -1486,6 +1646,9 @@
       <c r="F54" t="str">
         <v>Live</v>
       </c>
+      <c r="G54" t="str">
+        <v/>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="str">
@@ -1505,6 +1668,9 @@
       </c>
       <c r="F55" t="str">
         <v>Live</v>
+      </c>
+      <c r="G55" t="str">
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -1526,6 +1692,9 @@
       <c r="F56" t="str">
         <v>Live</v>
       </c>
+      <c r="G56" t="str">
+        <v/>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
@@ -1546,6 +1715,9 @@
       <c r="F57" t="str">
         <v>Live</v>
       </c>
+      <c r="G57" t="str">
+        <v/>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="str">
@@ -1566,6 +1738,9 @@
       <c r="F58" t="str">
         <v>Live</v>
       </c>
+      <c r="G58" t="str">
+        <v/>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="str">
@@ -1586,6 +1761,9 @@
       <c r="F59" t="str">
         <v>Live</v>
       </c>
+      <c r="G59" t="str">
+        <v/>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="str">
@@ -1606,6 +1784,9 @@
       <c r="F60" t="str">
         <v>Native build</v>
       </c>
+      <c r="G60" t="str">
+        <v/>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="str">
@@ -1625,6 +1806,9 @@
       </c>
       <c r="F61" t="str">
         <v>Live</v>
+      </c>
+      <c r="G61" t="str">
+        <v/>
       </c>
     </row>
     <row r="62">
@@ -1646,6 +1830,9 @@
       <c r="F62" t="str">
         <v>Live</v>
       </c>
+      <c r="G62" t="str">
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="str">
@@ -1666,6 +1853,9 @@
       <c r="F63" t="str">
         <v>Live</v>
       </c>
+      <c r="G63" t="str">
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -1686,6 +1876,9 @@
       <c r="F64" t="str">
         <v>Live</v>
       </c>
+      <c r="G64" t="str">
+        <v/>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -1706,6 +1899,9 @@
       <c r="F65" t="str">
         <v>Live</v>
       </c>
+      <c r="G65" t="str">
+        <v/>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -1725,6 +1921,9 @@
       </c>
       <c r="F66" t="str">
         <v>Live</v>
+      </c>
+      <c r="G66" t="str">
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -1746,6 +1945,9 @@
       <c r="F67" t="str">
         <v>Live</v>
       </c>
+      <c r="G67" t="str">
+        <v/>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -1766,6 +1968,9 @@
       <c r="F68" t="str">
         <v>Live</v>
       </c>
+      <c r="G68" t="str">
+        <v/>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -1786,6 +1991,9 @@
       <c r="F69" t="str">
         <v>Live</v>
       </c>
+      <c r="G69" t="str">
+        <v/>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -1806,6 +2014,9 @@
       <c r="F70" t="str">
         <v>Live</v>
       </c>
+      <c r="G70" t="str">
+        <v/>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -1826,6 +2037,9 @@
       <c r="F71" t="str">
         <v>Live</v>
       </c>
+      <c r="G71" t="str">
+        <v/>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -1846,6 +2060,9 @@
       <c r="F72" t="str">
         <v>Native build</v>
       </c>
+      <c r="G72" t="str">
+        <v/>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -1865,6 +2082,9 @@
       </c>
       <c r="F73" t="str">
         <v>Native build</v>
+      </c>
+      <c r="G73" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -1894,7 +2114,7 @@
     <mergeCell ref="B67:B73"/>
   </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G73"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>